<commit_message>
Report FPO import progress and derive parent FPO from WhatsApp uploader
</commit_message>
<xml_diff>
--- a/docs/fpo_leads_import_919372597458.xlsx
+++ b/docs/fpo_leads_import_919372597458.xlsx
@@ -64,9 +64,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,22 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:L4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,32 +416,29 @@
         <v>native_language</v>
       </c>
       <c r="F1" t="str">
-        <v>fpo_phone_number</v>
+        <v>address</v>
       </c>
       <c r="G1" t="str">
-        <v>address</v>
+        <v>village</v>
       </c>
       <c r="H1" t="str">
-        <v>village</v>
+        <v>district</v>
       </c>
       <c r="I1" t="str">
-        <v>district</v>
+        <v>state</v>
       </c>
       <c r="J1" t="str">
-        <v>state</v>
+        <v>pincode</v>
       </c>
       <c r="K1" t="str">
-        <v>pincode</v>
+        <v>latitude</v>
       </c>
       <c r="L1" t="str">
-        <v>latitude</v>
-      </c>
-      <c r="M1" t="str">
         <v>longitude</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="str">
+      <c r="A2" t="str">
         <v>919876543210</v>
       </c>
       <c r="B2" t="str">
@@ -472,33 +453,30 @@
       <c r="E2" t="str">
         <v>hindi</v>
       </c>
-      <c r="F2" s="1" t="str">
-        <v>919372597458</v>
+      <c r="F2" t="str">
+        <v>12 Market Road</v>
       </c>
       <c r="G2" t="str">
-        <v>12 Market Road</v>
+        <v>Kheda</v>
       </c>
       <c r="H2" t="str">
-        <v>Kheda</v>
+        <v>Indore</v>
       </c>
       <c r="I2" t="str">
-        <v>Indore</v>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="J2" t="str">
-        <v>Madhya Pradesh</v>
+        <v>452001</v>
       </c>
       <c r="K2" t="str">
-        <v>452001</v>
+        <v>22.7196</v>
       </c>
       <c r="L2" t="str">
-        <v>22.7196</v>
-      </c>
-      <c r="M2" t="str">
         <v>75.8577</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="str">
+      <c r="A3" t="str">
         <v>919876543211</v>
       </c>
       <c r="B3" t="str">
@@ -513,33 +491,30 @@
       <c r="E3" t="str">
         <v>english</v>
       </c>
-      <c r="F3" s="1" t="str">
-        <v>919372597458</v>
+      <c r="F3" t="str">
+        <v>45 Grain Market</v>
       </c>
       <c r="G3" t="str">
-        <v>45 Grain Market</v>
+        <v>Rau</v>
       </c>
       <c r="H3" t="str">
-        <v>Rau</v>
+        <v>Indore</v>
       </c>
       <c r="I3" t="str">
-        <v>Indore</v>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="J3" t="str">
-        <v>Madhya Pradesh</v>
+        <v>453331</v>
       </c>
       <c r="K3" t="str">
-        <v>453331</v>
+        <v>22.6840</v>
       </c>
       <c r="L3" t="str">
-        <v>22.6840</v>
-      </c>
-      <c r="M3" t="str">
         <v>75.8730</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="str">
+      <c r="A4" t="str">
         <v>919876543212</v>
       </c>
       <c r="B4" t="str">
@@ -554,34 +529,31 @@
       <c r="E4" t="str">
         <v>telugu</v>
       </c>
-      <c r="F4" s="1" t="str">
-        <v>919372597458</v>
+      <c r="F4" t="str">
+        <v>8 Farm Link Road</v>
       </c>
       <c r="G4" t="str">
-        <v>8 Farm Link Road</v>
+        <v>Dewas</v>
       </c>
       <c r="H4" t="str">
         <v>Dewas</v>
       </c>
       <c r="I4" t="str">
-        <v>Dewas</v>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="J4" t="str">
-        <v>Madhya Pradesh</v>
+        <v>455001</v>
       </c>
       <c r="K4" t="str">
-        <v>455001</v>
+        <v>22.9676</v>
       </c>
       <c r="L4" t="str">
-        <v>22.9676</v>
-      </c>
-      <c r="M4" t="str">
         <v>76.0534</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Start chatbots from any first text and validate FPO spreadsheet headers
</commit_message>
<xml_diff>
--- a/docs/fpo_leads_import_919372597458.xlsx
+++ b/docs/fpo_leads_import_919372597458.xlsx
@@ -397,7 +397,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,18 +437,21 @@
         <v>village</v>
       </c>
       <c r="H1" t="str">
+        <v>subdistrict</v>
+      </c>
+      <c r="I1" t="str">
         <v>district</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>state</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>pincode</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>latitude</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>longitude</v>
       </c>
     </row>
@@ -460,18 +478,21 @@
         <v>Kheda</v>
       </c>
       <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
         <v>Indore</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Madhya Pradesh</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>452001</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>22.7196</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>75.8577</v>
       </c>
     </row>
@@ -498,18 +519,21 @@
         <v>Rau</v>
       </c>
       <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
         <v>Indore</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>Madhya Pradesh</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>453331</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>22.6840</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>75.8730</v>
       </c>
     </row>
@@ -536,24 +560,27 @@
         <v>Dewas</v>
       </c>
       <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
         <v>Dewas</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Madhya Pradesh</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>455001</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>22.9676</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>76.0534</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>